<commit_message>
Washing sheet: keyboard navigation between days, update test
</commit_message>
<xml_diff>
--- a/frontend/static/templates/PM_Plant_Side_Template.xlsx
+++ b/frontend/static/templates/PM_Plant_Side_Template.xlsx
@@ -560,7 +560,7 @@
 5. Aux. Transformer (Aux. Transformer) — cycle days 14–15
 6. 4 Pole (4 Pole) — cycle days 16–17
 7. Earth pit (Earthing) — cycle days 18–19
-8. Miscellaneous (every other equipment type) — cycle days 20–22
+8. Miscellaneous (Street Light, ERT, … as one Miscellaneous job; any other equipment type not listed here) — cycle days 20–22
 9. Transmission line (Transmission line) — cycle days 23–24
 The GSS side (VCB, 4 Pole, Transmission line) follows after the plant side is finished.</t>
         </is>
@@ -694,7 +694,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Optional. How many units the plant has (ACCB-1 and ACCB-2 = 2). Blank = the plant's Unit configuration or Equipment Register.</t>
+          <t>Optional. How many units the plant has. Blank = the plant's Unit configuration or Equipment Register. ACCB Panel (ACCB-1 + ACCB-2) and Miscellaneous are always one job per plant.</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       <c r="B3" s="7" t="n"/>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>ACCB panel PM (ACCB-1, ACCB-2)</t>
+          <t>ACCB panel PM (ACCB-1 + ACCB-2, one job)</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -892,11 +892,11 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>1. Isolate. 2. Breaker operation check. 3. Busbar / terminal thermal scan. 4. Cable lugs. 5. Panel cleaning.</t>
+          <t>1. Isolate. 2. Breaker operation check. 3. Busbar / terminal thermal scan. 4. Cable lugs. 5. Panel cleaning. Do ACCB-1 and ACCB-2 in the same job.</t>
         </is>
       </c>
       <c r="I3" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" s="7" t="n"/>
       <c r="K3" s="8" t="n"/>
@@ -1149,13 +1149,13 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Transmission line</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Transmission line patrol &amp; PM (plant side)</t>
+          <t>Miscellaneous PM (Street Light, ERT, …)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1166,39 +1166,67 @@
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>PTW required</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>1. Line patrol. 2. Conductor / sag. 3. Insulators / jumpers. 4. Poles / towers. 5. Vegetation &amp; ROW.</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="n"/>
+          <t>1. Street Light. 2. ERT. 3. Any other small item at the plant. All in one job.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Plant side step 9 · cycle days 23–24</t>
+          <t>Plant side step 8 · cycle days 20–22</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Transmission line</t>
+        </is>
+      </c>
       <c r="B11" s="7" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Transmission line patrol &amp; PM (plant side)</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="8" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>PTW required</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>1. Line patrol. 2. Conductor / sag. 3. Insulators / jumpers. 4. Poles / towers. 5. Vegetation &amp; ROW.</t>
+        </is>
+      </c>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="8" t="n"/>
-      <c r="L11" s="9" t="n"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Plant side step 9 · cycle days 23–24</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -3849,7 +3877,7 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$A$2:$A$23</formula1>
+      <formula1>=Lists!$A$2:$A$24</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$B$2:$B$7</formula1>
@@ -3874,7 +3902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4006,96 +4034,103 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Transmission line</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Piling and Foundation</t>
+          <t>Transmission line</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WMS</t>
+          <t>Piling and Foundation</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OLTC(RTCC)</t>
+          <t>WMS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>OLTC(RTCC)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABT meters</t>
+          <t>RMS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>ABT meters</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CCTV</t>
+          <t>LA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Boundary wall</t>
+          <t>CCTV</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Water pipe line</t>
+          <t>Boundary wall</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vegetation</t>
+          <t>Water pipe line</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Vegetation</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BIKE</t>
+          <t>Street Light</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t>BIKE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
@@ -4112,7 +4147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4230,166 +4265,178 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Transmission line</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Line patrol  •  Conductor / sag inspection  •  Insulator / jumper inspection  •  Tower / pole / foundation inspection  •  Vegetation &amp; ROW clearance</t>
+          <t>Street Light, ERT and other small items — one job per plant</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Piling and Foundation</t>
+          <t>Transmission line</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Foundation inspection  •  Pile condition check  •  Settlement / alignment check  •  Crack / damage inspection  •  Corrective action review</t>
+          <t>Line patrol  •  Conductor / sag inspection  •  Insulator / jumper inspection  •  Tower / pole / foundation inspection  •  Vegetation &amp; ROW clearance</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WMS</t>
+          <t>Piling and Foundation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sensor cleaning  •  Irradiance / temperature sensor validation  •  Communication check  •  Calibration comparison  •  Mounting / cable inspection</t>
+          <t>Foundation inspection  •  Pile condition check  •  Settlement / alignment check  •  Crack / damage inspection  •  Corrective action review</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OLTC(RTCC)</t>
+          <t>WMS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tap-changer position / indication check  •  Auto-manual mode operation  •  Control wiring and relay inspection  •  Communication / SCADA signal check  •  Panel cleaning</t>
+          <t>Sensor cleaning  •  Irradiance / temperature sensor validation  •  Communication check  •  Calibration comparison  •  Mounting / cable inspection</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>OLTC(RTCC)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Communication availability  •  Data-gap / timestamp review  •  Router / modem / network check  •  Power / UPS backup check  •  Portal value validation</t>
+          <t>Tap-changer position / indication check  •  Auto-manual mode operation  •  Control wiring and relay inspection  •  Communication / SCADA signal check  •  Panel cleaning</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABT meters</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Meter reading validation  •  RTC / time sync  •  Seal / wiring inspection  •  Communication availability  •  Energy-data reconciliation</t>
+          <t>Communication availability  •  Data-gap / timestamp review  •  Router / modem / network check  •  Power / UPS backup check  •  Portal value validation</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>ABT meters</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Visual condition  •  Counter reading  •  Connection tightening  •  Earth continuity  •  Post-lightning inspection</t>
+          <t>Meter reading validation  •  RTC / time sync  •  Seal / wiring inspection  •  Communication availability  •  Energy-data reconciliation</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CCTV</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Camera feed check  •  Lens / housing cleaning  •  NVR / DVR recording &amp; storage check  •  UPS / network check  •  Coverage / night-vision verification</t>
+          <t>Visual condition  •  Counter reading  •  Connection tightening  •  Earth continuity  •  Post-lightning inspection</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Boundary wall</t>
+          <t>CCTV</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Wall / fencing patrol  •  Crack / settlement inspection  •  Gate / access check  •  Breach / damage repair review  •  Drainage / erosion observation</t>
+          <t>Camera feed check  •  Lens / housing cleaning  •  NVR / DVR recording &amp; storage check  •  UPS / network check  •  Coverage / night-vision verification</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Water pipe line</t>
+          <t>Boundary wall</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Leak / blockage inspection  •  Pump / valve operation  •  Pressure / flow observation  •  Joint / support inspection  •  Repair / flushing requirement</t>
+          <t>Wall / fencing patrol  •  Crack / settlement inspection  •  Gate / access check  •  Breach / damage repair review  •  Drainage / erosion observation</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vegetation</t>
+          <t>Water pipe line</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Grass / weed cutting  •  Module shading check  •  Fire-risk / dry biomass removal  •  ROW / access clearing  •  Waste disposal</t>
+          <t>Leak / blockage inspection  •  Pump / valve operation  •  Pressure / flow observation  •  Joint / support inspection  •  Repair / flushing requirement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Vegetation</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fixture operation  •  Timer / controller check  •  Cable / pole inspection  •  Earthing check  •  Night operation verification</t>
+          <t>Grass / weed cutting  •  Module shading check  •  Fire-risk / dry biomass removal  •  ROW / access clearing  •  Waste disposal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BIKE</t>
+          <t>Street Light</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bike Not Starting  •  Accident / Body Damage  •  Functional check  •  Engine Problem  •  Corrective action review</t>
+          <t>Fixture operation  •  Timer / controller check  •  Cable / pole inspection  •  Earthing check  •  Night operation verification</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>BIKE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bike Not Starting  •  Accident / Body Damage  •  Functional check  •  Engine Problem  •  Corrective action review</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Define task-specific checklist  •  Capture measurements / readings  •  Attach photo / video evidence  •  Record remarks / anomalies  •  Escalate problem to Issue if required</t>
         </is>

</xml_diff>

<commit_message>
PM: cycle panel, all cycle equipment in Plants grid with add buttons; Excel templates updated; washing compliance as percentage per cycle
</commit_message>
<xml_diff>
--- a/frontend/static/templates/PM_Plant_Side_Template.xlsx
+++ b/frontend/static/templates/PM_Plant_Side_Template.xlsx
@@ -4242,7 +4242,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Incomer / outgoing breaker operation, busbar / terminal thermal scan, cable lugs, panel cleaning</t>
+          <t>Incomer / outgoing breaker operation  ·  Busbar / terminal thermal scan  ·  Cable / lug tightening  ·  Indication / metering check  ·  Panel cleaning</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Street Light, ERT and other small items — one job per plant; list them in Remarks</t>
+          <t>One job per plant for the small items: Street Light  ·  ERT  ·  any other item. Name the items in Remarks.</t>
         </is>
       </c>
     </row>

</xml_diff>